<commit_message>
dev-auto-content: update the initial sheets with the values from the filtered sheet
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T1_Analysis.xlsx
+++ b/Ref_Files/Test_Excell_T1_Analysis.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Analysys" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Analysis" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -530,9 +530,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>628200</xdr:colOff>
+      <xdr:colOff>627840</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>314640</xdr:rowOff>
+      <xdr:rowOff>314280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -546,7 +546,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5784840" y="31320"/>
-          <a:ext cx="1261800" cy="283320"/>
+          <a:ext cx="1261440" cy="282960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -744,7 +744,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -769,7 +769,7 @@
       <c r="G2" s="4"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="3"/>
@@ -779,7 +779,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
@@ -803,7 +803,7 @@
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -827,7 +827,7 @@
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -837,7 +837,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
@@ -847,7 +847,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>15</v>
       </c>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
@@ -1106,7 +1106,7 @@
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
         <v>31</v>
       </c>
@@ -1303,7 +1303,7 @@
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
     </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
         <v>33</v>
       </c>
@@ -1315,7 +1315,7 @@
       <c r="G40" s="8"/>
       <c r="H40" s="2"/>
     </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
         <v>34</v>
       </c>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="H41" s="2"/>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
@@ -1339,7 +1339,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11"/>
       <c r="B43" s="11" t="s">
         <v>19</v>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="H43" s="2"/>
     </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H44" s="2"/>
     </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="3"/>
@@ -1387,7 +1387,7 @@
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
     </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11"/>
       <c r="B46" s="11" t="s">
         <v>23</v>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="H46" s="2"/>
     </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="H47" s="2"/>
     </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="3"/>
@@ -1437,7 +1437,7 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
     </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11"/>
       <c r="B49" s="11" t="s">
         <v>26</v>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="H49" s="2"/>
     </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="H50" s="2"/>
     </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
         <v>20</v>
       </c>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="H51" s="2"/>
     </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="3"/>
@@ -1501,7 +1501,7 @@
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
     </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11"/>
       <c r="B53" s="11" t="s">
         <v>7</v>
@@ -1513,7 +1513,7 @@
       <c r="G53" s="11"/>
       <c r="H53" s="2"/>
     </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
         <v>29</v>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="H54" s="2"/>
     </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2"/>
       <c r="B55" s="2" t="s">
         <v>30</v>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H55" s="2"/>
     </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
       <c r="B56" s="2" t="s">
         <v>36</v>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2"/>
       <c r="B57" s="2" t="s">
         <v>37</v>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="H57" s="2"/>
     </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="3"/>
@@ -1583,7 +1583,7 @@
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
     </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8"/>
       <c r="B59" s="8" t="s">
         <v>7</v>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H59" s="2"/>
     </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="3"/>
@@ -1607,7 +1607,7 @@
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
     </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
         <v>38</v>
       </c>
@@ -1619,7 +1619,7 @@
       <c r="G61" s="8"/>
       <c r="H61" s="2"/>
     </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
         <v>39</v>
       </c>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="H62" s="2"/>
     </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="3"/>
@@ -1643,7 +1643,7 @@
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
     </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11"/>
       <c r="B64" s="11" t="s">
         <v>19</v>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="H64" s="2"/>
     </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
         <v>20</v>
       </c>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H65" s="2"/>
     </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
         <v>20</v>
       </c>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="H66" s="2"/>
     </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="3"/>
@@ -1715,7 +1715,7 @@
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
     </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2"/>
       <c r="B68" s="11" t="s">
         <v>23</v>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="H68" s="2"/>
     </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
@@ -1741,7 +1741,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2"/>
       <c r="B70" s="11" t="s">
         <v>26</v>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="H70" s="2"/>
     </row>
-    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
       <c r="B71" s="2" t="s">
         <v>35</v>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="H71" s="2"/>
     </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="3"/>
@@ -1783,7 +1783,7 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
     </row>
-    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2"/>
       <c r="B73" s="11" t="s">
         <v>7</v>
@@ -1795,7 +1795,7 @@
       <c r="G73" s="11"/>
       <c r="H73" s="2"/>
     </row>
-    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="11"/>
       <c r="B74" s="2" t="s">
         <v>29</v>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H74" s="2"/>
     </row>
-    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="3"/>
@@ -1819,7 +1819,7 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
     </row>
-    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="3"/>
@@ -1829,7 +1829,7 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
     </row>
-    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8"/>
       <c r="B77" s="8" t="s">
         <v>7</v>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="H77" s="2"/>
     </row>
-    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="3"/>
@@ -1853,7 +1853,7 @@
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
     </row>
-    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="s">
         <v>42</v>
       </c>
@@ -1865,7 +1865,7 @@
       <c r="G79" s="8"/>
       <c r="H79" s="2"/>
     </row>
-    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="11" t="s">
         <v>43</v>
       </c>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="H80" s="2"/>
     </row>
-    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="3"/>
@@ -1889,7 +1889,7 @@
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
     </row>
-    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="11"/>
       <c r="B82" s="11" t="s">
         <v>19</v>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="H82" s="2"/>
     </row>
-    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -1913,7 +1913,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2"/>
       <c r="B84" s="11" t="s">
         <v>23</v>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="H84" s="2"/>
     </row>
-    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2"/>
       <c r="B85" s="2" t="s">
         <v>24</v>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="H85" s="2"/>
     </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2"/>
       <c r="B86" s="2" t="s">
         <v>45</v>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H86" s="2"/>
     </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="3"/>
@@ -1975,7 +1975,7 @@
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
     </row>
-    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2"/>
       <c r="B88" s="11" t="s">
         <v>7</v>
@@ -1987,7 +1987,7 @@
       <c r="G88" s="11"/>
       <c r="H88" s="2"/>
     </row>
-    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="3"/>
@@ -1997,7 +1997,7 @@
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
     </row>
-    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8"/>
       <c r="B90" s="8" t="s">
         <v>7</v>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="H90" s="2"/>
     </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
@@ -2021,7 +2021,7 @@
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
     </row>
-    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="s">
         <v>46</v>
       </c>
@@ -2033,7 +2033,7 @@
       <c r="G92" s="8"/>
       <c r="H92" s="2"/>
     </row>
-    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
         <v>47</v>
       </c>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="H93" s="2"/>
     </row>
-    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
@@ -2057,7 +2057,7 @@
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
     </row>
-    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11"/>
       <c r="B95" s="11" t="s">
         <v>19</v>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="H95" s="2"/>
     </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
         <v>20</v>
       </c>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="H96" s="2"/>
     </row>
-    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
         <v>20</v>
       </c>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="H97" s="2"/>
     </row>
-    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2"/>
       <c r="B98" s="2" t="s">
         <v>48</v>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="H98" s="2"/>
     </row>
-    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2"/>
       <c r="B99" s="2" t="s">
         <v>49</v>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="H99" s="2"/>
     </row>
-    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="3"/>
@@ -2173,7 +2173,7 @@
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
     </row>
-    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2"/>
       <c r="B101" s="11" t="s">
         <v>23</v>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="H101" s="2"/>
     </row>
-    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2"/>
       <c r="B102" s="2" t="s">
         <v>24</v>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="H102" s="2"/>
     </row>
-    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="3"/>
@@ -2217,7 +2217,7 @@
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
     </row>
-    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2"/>
       <c r="B104" s="11" t="s">
         <v>26</v>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="H104" s="2"/>
     </row>
-    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2"/>
       <c r="B105" s="2" t="s">
         <v>27</v>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="H105" s="2"/>
     </row>
-    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="3"/>
@@ -2259,7 +2259,7 @@
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
     </row>
-    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2"/>
       <c r="B107" s="11" t="s">
         <v>7</v>
@@ -2271,7 +2271,7 @@
       <c r="G107" s="11"/>
       <c r="H107" s="2"/>
     </row>
-    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="11"/>
       <c r="B108" s="2" t="s">
         <v>29</v>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="H108" s="2"/>
     </row>
-    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="11"/>
       <c r="B109" s="2" t="s">
         <v>30</v>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="H109" s="2"/>
     </row>
-    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="11"/>
       <c r="B110" s="2" t="s">
         <v>36</v>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="H110" s="2"/>
     </row>
-    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="11"/>
       <c r="B111" s="2" t="s">
         <v>37</v>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="H111" s="2"/>
     </row>
-    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="3"/>
@@ -2337,7 +2337,7 @@
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
     </row>
-    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8"/>
       <c r="B113" s="8" t="s">
         <v>7</v>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="H113" s="2"/>
     </row>
-    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="3"/>
@@ -2361,7 +2361,7 @@
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
     </row>
-    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="8" t="s">
         <v>50</v>
       </c>
@@ -2373,7 +2373,7 @@
       <c r="G115" s="8"/>
       <c r="H115" s="2"/>
     </row>
-    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="11" t="s">
         <v>51</v>
       </c>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H116" s="2"/>
     </row>
-    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="3"/>
@@ -2397,7 +2397,7 @@
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
     </row>
-    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="11"/>
       <c r="B118" s="11" t="s">
         <v>19</v>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="H118" s="2"/>
     </row>
-    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="3"/>
@@ -2421,7 +2421,7 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
     </row>
-    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2"/>
       <c r="B120" s="11" t="s">
         <v>23</v>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H120" s="2"/>
     </row>
-    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="3"/>
@@ -2447,7 +2447,7 @@
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
     </row>
-    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2"/>
       <c r="B122" s="11" t="s">
         <v>26</v>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="H122" s="2"/>
     </row>
-    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="3"/>
@@ -2471,7 +2471,7 @@
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
     </row>
-    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2"/>
       <c r="B124" s="11" t="s">
         <v>7</v>
@@ -2483,7 +2483,7 @@
       <c r="G124" s="11"/>
       <c r="H124" s="2"/>
     </row>
-    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="3"/>
@@ -2493,7 +2493,7 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
     </row>
-    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="8"/>
       <c r="B126" s="8" t="s">
         <v>7</v>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H126" s="2"/>
     </row>
-    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="3"/>
@@ -2517,7 +2517,7 @@
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
     </row>
-    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="8" t="s">
         <v>52</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="G128" s="8"/>
       <c r="H128" s="2"/>
     </row>
-    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
         <v>53</v>
       </c>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H129" s="2"/>
     </row>
-    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="3"/>
@@ -2553,7 +2553,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="11"/>
       <c r="B131" s="11" t="s">
         <v>19</v>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="H131" s="2"/>
     </row>
-    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="3"/>
@@ -2577,7 +2577,7 @@
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
     </row>
-    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2"/>
       <c r="B133" s="11" t="s">
         <v>23</v>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="H133" s="2"/>
     </row>
-    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2"/>
       <c r="B134" s="2" t="s">
         <v>24</v>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="H134" s="2"/>
     </row>
-    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2"/>
       <c r="B135" s="2" t="s">
         <v>45</v>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="H135" s="2"/>
     </row>
-    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="3"/>
@@ -2635,7 +2635,7 @@
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
     </row>
-    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2"/>
       <c r="B137" s="11" t="s">
         <v>26</v>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="H137" s="2"/>
     </row>
-    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="3"/>
@@ -2659,7 +2659,7 @@
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
     </row>
-    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2"/>
       <c r="B139" s="11" t="s">
         <v>7</v>
@@ -2671,7 +2671,7 @@
       <c r="G139" s="11"/>
       <c r="H139" s="2"/>
     </row>
-    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2"/>
       <c r="B140" s="2" t="s">
         <v>29</v>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="H140" s="2"/>
     </row>
-    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="3"/>
@@ -2695,7 +2695,7 @@
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
     </row>
-    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="8"/>
       <c r="B142" s="8" t="s">
         <v>7</v>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="H142" s="2"/>
     </row>
-    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="3"/>
@@ -2719,7 +2719,7 @@
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
     </row>
-    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="8" t="s">
         <v>54</v>
       </c>
@@ -2731,7 +2731,7 @@
       <c r="G144" s="8"/>
       <c r="H144" s="2"/>
     </row>
-    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
         <v>55</v>
       </c>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H145" s="2"/>
     </row>
-    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="3"/>
@@ -2755,7 +2755,7 @@
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
     </row>
-    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="11"/>
       <c r="B147" s="11" t="s">
         <v>19</v>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="H147" s="2"/>
     </row>
-    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2"/>
       <c r="B148" s="2" t="s">
         <v>21</v>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="H148" s="2"/>
     </row>
-    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2"/>
       <c r="B149" s="2" t="s">
         <v>41</v>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H149" s="2"/>
     </row>
-    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2"/>
       <c r="B150" s="2" t="s">
         <v>48</v>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="H150" s="2"/>
     </row>
-    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="3"/>
@@ -2827,7 +2827,7 @@
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
     </row>
-    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2"/>
       <c r="B152" s="11" t="s">
         <v>23</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H152" s="2"/>
     </row>
-    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2"/>
       <c r="B153" s="2" t="s">
         <v>24</v>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="H153" s="2"/>
     </row>
-    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="3"/>
@@ -2869,7 +2869,7 @@
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
     </row>
-    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2"/>
       <c r="B155" s="11" t="s">
         <v>26</v>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="H155" s="2"/>
     </row>
-    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2"/>
       <c r="B156" s="2" t="s">
         <v>45</v>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="H156" s="2"/>
     </row>
-    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="3"/>
@@ -2909,7 +2909,7 @@
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
     </row>
-    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2"/>
       <c r="B158" s="11" t="s">
         <v>7</v>
@@ -2921,7 +2921,7 @@
       <c r="G158" s="11"/>
       <c r="H158" s="2"/>
     </row>
-    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2"/>
       <c r="B159" s="2" t="s">
         <v>29</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="H159" s="2"/>
     </row>
-    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="3"/>
@@ -2945,7 +2945,7 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
     </row>
-    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="8"/>
       <c r="B161" s="8" t="s">
         <v>7</v>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="H161" s="2"/>
     </row>
-    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="3"/>
@@ -2969,7 +2969,7 @@
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
     </row>
-    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="8" t="s">
         <v>56</v>
       </c>
@@ -2981,7 +2981,7 @@
       <c r="G163" s="8"/>
       <c r="H163" s="2"/>
     </row>
-    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="11" t="s">
         <v>57</v>
       </c>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="H164" s="2"/>
     </row>
-    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="3"/>
@@ -3005,7 +3005,7 @@
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
     </row>
-    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="11"/>
       <c r="B166" s="11" t="s">
         <v>19</v>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="H166" s="2"/>
     </row>
-    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
         <v>20</v>
       </c>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="H167" s="2"/>
     </row>
-    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="3"/>
@@ -3053,7 +3053,7 @@
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
     </row>
-    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2"/>
       <c r="B169" s="11" t="s">
         <v>23</v>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="H169" s="2"/>
     </row>
-    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2"/>
       <c r="B170" s="2" t="s">
         <v>24</v>
@@ -3087,7 +3087,7 @@
       </c>
       <c r="H170" s="2"/>
     </row>
-    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2"/>
       <c r="B171" s="2" t="s">
         <v>45</v>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="H171" s="2"/>
     </row>
-    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="3"/>
@@ -3115,7 +3115,7 @@
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
     </row>
-    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2"/>
       <c r="B173" s="11" t="s">
         <v>26</v>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="H173" s="2"/>
     </row>
-    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2"/>
       <c r="B174" s="2" t="s">
         <v>27</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="H174" s="2"/>
     </row>
-    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="3"/>
@@ -3157,7 +3157,7 @@
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
     </row>
-    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2"/>
       <c r="B176" s="11" t="s">
         <v>7</v>
@@ -3169,7 +3169,7 @@
       <c r="G176" s="11"/>
       <c r="H176" s="2"/>
     </row>
-    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="11"/>
       <c r="B177" s="2" t="s">
         <v>29</v>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="H177" s="2"/>
     </row>
-    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="11"/>
       <c r="B178" s="2" t="s">
         <v>30</v>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H178" s="2"/>
     </row>
-    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="3"/>
@@ -3207,7 +3207,7 @@
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
     </row>
-    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="8"/>
       <c r="B180" s="8" t="s">
         <v>7</v>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="H180" s="2"/>
     </row>
-    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="3"/>
@@ -3231,7 +3231,7 @@
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
     </row>
-    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="8" t="s">
         <v>58</v>
       </c>
@@ -3243,7 +3243,7 @@
       <c r="G182" s="8"/>
       <c r="H182" s="2"/>
     </row>
-    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="11" t="s">
         <v>59</v>
       </c>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="H183" s="2"/>
     </row>
-    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="3"/>
@@ -3267,7 +3267,7 @@
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
     </row>
-    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="11"/>
       <c r="B185" s="11" t="s">
         <v>19</v>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H185" s="2"/>
     </row>
-    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2"/>
       <c r="B186" s="2" t="s">
         <v>21</v>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="H186" s="2"/>
     </row>
-    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -3307,7 +3307,7 @@
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
     </row>
-    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2"/>
       <c r="B188" s="11" t="s">
         <v>23</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H188" s="2"/>
     </row>
-    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2"/>
       <c r="B189" s="2" t="s">
         <v>24</v>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="H189" s="2"/>
     </row>
-    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="3"/>
@@ -3349,7 +3349,7 @@
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
     </row>
-    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2"/>
       <c r="B191" s="11" t="s">
         <v>26</v>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="H191" s="2"/>
     </row>
-    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="2"/>
       <c r="B192" s="2" t="s">
         <v>27</v>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="H192" s="2"/>
     </row>
-    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="3"/>
@@ -3389,7 +3389,7 @@
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
     </row>
-    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="2"/>
       <c r="B194" s="11" t="s">
         <v>7</v>
@@ -3401,7 +3401,7 @@
       <c r="G194" s="11"/>
       <c r="H194" s="2"/>
     </row>
-    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="2"/>
       <c r="B195" s="2" t="s">
         <v>29</v>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="H195" s="2"/>
     </row>
-    <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="3"/>
@@ -3425,7 +3425,7 @@
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
     </row>
-    <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="8"/>
       <c r="B197" s="8" t="s">
         <v>7</v>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="H197" s="2"/>
     </row>
-    <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="3"/>
@@ -3449,7 +3449,7 @@
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
     </row>
-    <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="8" t="s">
         <v>60</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="G199" s="8"/>
       <c r="H199" s="2"/>
     </row>
-    <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="11" t="s">
         <v>61</v>
       </c>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="H200" s="2"/>
     </row>
-    <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
       <c r="C201" s="3"/>
@@ -3485,7 +3485,7 @@
       <c r="G201" s="2"/>
       <c r="H201" s="2"/>
     </row>
-    <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="2"/>
       <c r="B202" s="11" t="s">
         <v>23</v>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="H202" s="2"/>
     </row>
-    <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="2"/>
       <c r="B203" s="2" t="s">
         <v>24</v>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="H203" s="2"/>
     </row>
-    <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
       <c r="C204" s="3"/>
@@ -3527,7 +3527,7 @@
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
     </row>
-    <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="2"/>
       <c r="B205" s="11" t="s">
         <v>7</v>
@@ -3539,7 +3539,7 @@
       <c r="G205" s="11"/>
       <c r="H205" s="2"/>
     </row>
-    <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="2"/>
       <c r="B206" s="2" t="s">
         <v>29</v>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="H206" s="2"/>
     </row>
-    <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="2"/>
       <c r="B207" s="2"/>
       <c r="C207" s="3"/>
@@ -3563,7 +3563,7 @@
       <c r="G207" s="2"/>
       <c r="H207" s="2"/>
     </row>
-    <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="8"/>
       <c r="B208" s="8" t="s">
         <v>7</v>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="H208" s="2"/>
     </row>
-    <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="2"/>
       <c r="B209" s="2"/>
       <c r="C209" s="3"/>
@@ -3587,7 +3587,7 @@
       <c r="G209" s="2"/>
       <c r="H209" s="2"/>
     </row>
-    <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="8" t="s">
         <v>63</v>
       </c>
@@ -3599,7 +3599,7 @@
       <c r="G210" s="8"/>
       <c r="H210" s="2"/>
     </row>
-    <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="11" t="s">
         <v>64</v>
       </c>
@@ -3613,7 +3613,7 @@
       </c>
       <c r="H211" s="2"/>
     </row>
-    <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="2"/>
       <c r="B212" s="2"/>
       <c r="C212" s="3"/>
@@ -3623,7 +3623,7 @@
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
     </row>
-    <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="11"/>
       <c r="B213" s="11" t="s">
         <v>19</v>
@@ -3637,7 +3637,7 @@
       </c>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="2"/>
       <c r="B214" s="2" t="s">
         <v>21</v>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="H214" s="2"/>
     </row>
-    <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="2"/>
       <c r="B215" s="2" t="s">
         <v>41</v>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="H215" s="2"/>
     </row>
-    <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="2"/>
       <c r="B216" s="2"/>
       <c r="C216" s="3"/>
@@ -3679,7 +3679,7 @@
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
     </row>
-    <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="2"/>
       <c r="B217" s="11" t="s">
         <v>23</v>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="H217" s="2"/>
     </row>
-    <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="2"/>
       <c r="B218" s="2" t="s">
         <v>24</v>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="H218" s="2"/>
     </row>
-    <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="2"/>
       <c r="B219" s="2" t="s">
         <v>45</v>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="H219" s="2"/>
     </row>
-    <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="2"/>
       <c r="B220" s="2" t="s">
         <v>65</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="H220" s="2"/>
     </row>
-    <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="2"/>
       <c r="B221" s="2"/>
       <c r="C221" s="3"/>
@@ -3753,7 +3753,7 @@
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
     </row>
-    <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="2"/>
       <c r="B222" s="11" t="s">
         <v>26</v>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="H222" s="2"/>
     </row>
-    <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="2"/>
       <c r="B223" s="2" t="s">
         <v>27</v>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="H223" s="2"/>
     </row>
-    <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="2"/>
       <c r="B224" s="2"/>
       <c r="C224" s="3"/>
@@ -3793,7 +3793,7 @@
       <c r="G224" s="2"/>
       <c r="H224" s="2"/>
     </row>
-    <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="2"/>
       <c r="B225" s="11" t="s">
         <v>7</v>
@@ -3805,7 +3805,7 @@
       <c r="G225" s="11"/>
       <c r="H225" s="2"/>
     </row>
-    <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="2"/>
       <c r="B226" s="2" t="s">
         <v>29</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="H226" s="2"/>
     </row>
-    <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="2"/>
       <c r="B227" s="2"/>
       <c r="C227" s="3"/>
@@ -3829,7 +3829,7 @@
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
     </row>
-    <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="8"/>
       <c r="B228" s="8" t="s">
         <v>7</v>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H228" s="2"/>
     </row>
-    <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="2"/>
       <c r="B229" s="2"/>
       <c r="C229" s="3"/>
@@ -3853,7 +3853,7 @@
       <c r="G229" s="2"/>
       <c r="H229" s="2"/>
     </row>
-    <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="8" t="s">
         <v>66</v>
       </c>
@@ -3865,7 +3865,7 @@
       <c r="G230" s="8"/>
       <c r="H230" s="2"/>
     </row>
-    <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="11" t="s">
         <v>67</v>
       </c>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="H231" s="2"/>
     </row>
-    <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="2"/>
       <c r="B232" s="2"/>
       <c r="C232" s="3"/>
@@ -3889,7 +3889,7 @@
       <c r="G232" s="2"/>
       <c r="H232" s="2"/>
     </row>
-    <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="2"/>
       <c r="B233" s="11" t="s">
         <v>23</v>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="H233" s="2"/>
     </row>
-    <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="2"/>
       <c r="B234" s="2" t="s">
         <v>24</v>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="H234" s="2"/>
     </row>
-    <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="2"/>
       <c r="B235" s="2"/>
       <c r="C235" s="3"/>
@@ -3931,7 +3931,7 @@
       <c r="G235" s="2"/>
       <c r="H235" s="2"/>
     </row>
-    <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="2"/>
       <c r="B236" s="11" t="s">
         <v>7</v>
@@ -3943,7 +3943,7 @@
       <c r="G236" s="11"/>
       <c r="H236" s="2"/>
     </row>
-    <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="2"/>
       <c r="B237" s="2" t="s">
         <v>29</v>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="H237" s="2"/>
     </row>
-    <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="2"/>
       <c r="B238" s="2" t="s">
         <v>30</v>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="H238" s="2"/>
     </row>
-    <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="2"/>
       <c r="B239" s="2" t="s">
         <v>36</v>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="H239" s="2"/>
     </row>
-    <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="2"/>
       <c r="B240" s="2" t="s">
         <v>37</v>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="H240" s="2"/>
     </row>
-    <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="2"/>
       <c r="B241" s="2"/>
       <c r="C241" s="3"/>
@@ -4009,7 +4009,7 @@
       <c r="G241" s="2"/>
       <c r="H241" s="2"/>
     </row>
-    <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="8"/>
       <c r="B242" s="8" t="s">
         <v>7</v>
@@ -4033,7 +4033,7 @@
       <c r="G243" s="2"/>
       <c r="H243" s="2"/>
     </row>
-    <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="8" t="s">
         <v>68</v>
       </c>
@@ -4198,7 +4198,7 @@
       <c r="G255" s="2"/>
       <c r="H255" s="2"/>
     </row>
-    <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="8" t="s">
         <v>70</v>
       </c>
@@ -4439,7 +4439,7 @@
       <c r="G271" s="2"/>
       <c r="H271" s="2"/>
     </row>
-    <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="8" t="s">
         <v>72</v>
       </c>
@@ -4451,7 +4451,7 @@
       <c r="G272" s="8"/>
       <c r="H272" s="2"/>
     </row>
-    <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="11" t="s">
         <v>73</v>
       </c>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="H273" s="2"/>
     </row>
-    <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="2"/>
       <c r="B274" s="2"/>
       <c r="C274" s="3"/>
@@ -4475,7 +4475,7 @@
       <c r="G274" s="2"/>
       <c r="H274" s="2"/>
     </row>
-    <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="11"/>
       <c r="B275" s="11" t="s">
         <v>19</v>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="H275" s="2"/>
     </row>
-    <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="2" t="s">
         <v>20</v>
       </c>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="H276" s="2"/>
     </row>
-    <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="2"/>
       <c r="B277" s="2" t="s">
         <v>41</v>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="H277" s="2"/>
     </row>
-    <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="2"/>
       <c r="B278" s="2"/>
       <c r="C278" s="3"/>
@@ -4545,7 +4545,7 @@
       <c r="G278" s="2"/>
       <c r="H278" s="2"/>
     </row>
-    <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="2"/>
       <c r="B279" s="11" t="s">
         <v>23</v>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H279" s="2"/>
     </row>
-    <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="2"/>
       <c r="B280" s="2" t="s">
         <v>24</v>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H280" s="2"/>
     </row>
-    <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="2"/>
       <c r="B281" s="2" t="s">
         <v>45</v>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="H281" s="2"/>
     </row>
-    <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="2"/>
       <c r="B282" s="2"/>
       <c r="C282" s="3"/>
@@ -4607,7 +4607,7 @@
       <c r="G282" s="2"/>
       <c r="H282" s="2"/>
     </row>
-    <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="8"/>
       <c r="B283" s="8" t="s">
         <v>7</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="H283" s="2"/>
     </row>
-    <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="2"/>
       <c r="B284" s="2"/>
       <c r="C284" s="3"/>
@@ -4631,7 +4631,7 @@
       <c r="G284" s="2"/>
       <c r="H284" s="2"/>
     </row>
-    <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="2"/>
       <c r="B285" s="2"/>
       <c r="C285" s="3"/>
@@ -4641,7 +4641,7 @@
       <c r="G285" s="2"/>
       <c r="H285" s="2"/>
     </row>
-    <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="2"/>
       <c r="B286" s="2"/>
       <c r="C286" s="3"/>
@@ -4651,7 +4651,7 @@
       <c r="G286" s="2"/>
       <c r="H286" s="2"/>
     </row>
-    <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="2"/>
       <c r="B287" s="2"/>
       <c r="C287" s="3"/>
@@ -4661,7 +4661,7 @@
       <c r="G287" s="2"/>
       <c r="H287" s="2"/>
     </row>
-    <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="2" t="s">
         <v>74</v>
       </c>
@@ -4673,7 +4673,7 @@
       <c r="G288" s="2"/>
       <c r="H288" s="2"/>
     </row>
-    <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="2"/>
       <c r="B289" s="2" t="s">
         <v>75</v>
@@ -4685,7 +4685,7 @@
       <c r="G289" s="2"/>
       <c r="H289" s="2"/>
     </row>
-    <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="2"/>
       <c r="B290" s="2"/>
       <c r="C290" s="3"/>
@@ -4695,7 +4695,7 @@
       <c r="G290" s="2"/>
       <c r="H290" s="2"/>
     </row>
-    <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="2" t="s">
         <v>76</v>
       </c>
@@ -4707,7 +4707,7 @@
       <c r="G291" s="2"/>
       <c r="H291" s="2"/>
     </row>
-    <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="2"/>
       <c r="B292" s="2" t="s">
         <v>77</v>

</xml_diff>